<commit_message>
MITRE: tool-native coverage overlay design plan + template guidance
docs/planning/MITRE_TOOL_COVERAGE_PLAN.md — the durable answer to 'our
EDR covers that TTP': client declares tools, assessment overlays the
techniques those tools were evaluated as detecting (MITRE ATT&CK
Evaluations, cited), always as a second labeled number, never merged
into the rule-based score. T1 backend core + T2 surfaces pending.

Environment template updated ahead of the feature: Security Tooling
sheet gains a Notes column and canonical product-name examples
(CrowdStrike Falcon, Microsoft Defender for Endpoint, …); Read Me
explains precise names power both roadmap tiers and the coming overlay.
Verified the sheet still parses clean (header not ingested as an entry).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/mitre-environment-template.xlsx
+++ b/apps/web/public/templates/mitre-environment-template.xlsx
@@ -527,10 +527,10 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Security Tooling -- products you own but may not have onboarded for logging yet. Used for the next-tier "onboard this, then detect" gaps.</t>
+          <t>Security Tooling -- every security product you run (EDR, email, identity, network), one per row, using the precise product name (e.g. "CrowdStrike Falcon", "Microsoft Defender for Endpoint"). Used two ways: "onboard this, then detect" roadmap tiers today, and tool-native detection credit (from MITRE ATT&amp;CK Evaluations results) as that feature lands -- exact names make both work.</t>
         </is>
       </c>
     </row>
@@ -1738,10 +1738,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A103"/>
+  <dimension ref="A1:B105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1750,320 +1751,455 @@
           <t>Tool</t>
         </is>
       </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Notes (optional)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>CrowdStrike Falcon EDR</t>
+          <t>CrowdStrike Falcon</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>EDR on all workstations + servers</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
+          <t>Microsoft Defender for Endpoint</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>servers only</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
           <t>Proofpoint Email Security</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Okta</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>workforce identity</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n"/>
+      <c r="B30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
+      <c r="B31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
+      <c r="B32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
+      <c r="B33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
+      <c r="B34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
+      <c r="B35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
+      <c r="B36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
+      <c r="B37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
+      <c r="B38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
+      <c r="B39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
+      <c r="B40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
+      <c r="B41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
+      <c r="B42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
+      <c r="B43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
+      <c r="B44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n"/>
+      <c r="B45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n"/>
+      <c r="B46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>
+      <c r="B47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n"/>
+      <c r="B48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n"/>
+      <c r="B49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>
+      <c r="B50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n"/>
+      <c r="B51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>
+      <c r="B52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>
+      <c r="B53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
+      <c r="B54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
+      <c r="B55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n"/>
+      <c r="B56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n"/>
+      <c r="B57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n"/>
+      <c r="B58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n"/>
+      <c r="B59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="n"/>
+      <c r="B60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="n"/>
+      <c r="B61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="6" t="n"/>
+      <c r="B62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n"/>
+      <c r="B63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="6" t="n"/>
+      <c r="B64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n"/>
+      <c r="B65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n"/>
+      <c r="B66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="n"/>
+      <c r="B67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="n"/>
+      <c r="B68" s="6" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n"/>
+      <c r="B69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="6" t="n"/>
+      <c r="B70" s="6" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n"/>
+      <c r="B71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="n"/>
+      <c r="B72" s="6" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n"/>
+      <c r="B73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n"/>
+      <c r="B74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n"/>
+      <c r="B75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="6" t="n"/>
+      <c r="B76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="n"/>
+      <c r="B77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n"/>
+      <c r="B78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="n"/>
+      <c r="B79" s="6" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="6" t="n"/>
+      <c r="B80" s="6" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="n"/>
+      <c r="B81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n"/>
+      <c r="B82" s="6" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="n"/>
+      <c r="B83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="6" t="n"/>
+      <c r="B84" s="6" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="n"/>
+      <c r="B85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="6" t="n"/>
+      <c r="B86" s="6" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="n"/>
+      <c r="B87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="6" t="n"/>
+      <c r="B88" s="6" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n"/>
+      <c r="B89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="6" t="n"/>
+      <c r="B90" s="6" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="6" t="n"/>
+      <c r="B91" s="6" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="6" t="n"/>
+      <c r="B92" s="6" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="6" t="n"/>
+      <c r="B93" s="6" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="6" t="n"/>
+      <c r="B94" s="6" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="n"/>
+      <c r="B95" s="6" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="6" t="n"/>
+      <c r="B96" s="6" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="6" t="n"/>
+      <c r="B97" s="6" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="6" t="n"/>
+      <c r="B98" s="6" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="6" t="n"/>
+      <c r="B99" s="6" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="6" t="n"/>
+      <c r="B100" s="6" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="6" t="n"/>
+      <c r="B101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="6" t="n"/>
+      <c r="B102" s="6" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="6" t="n"/>
+      <c r="B103" s="6" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="n"/>
+      <c r="B104" s="6" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="n"/>
+      <c r="B105" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>